<commit_message>
Choses the hyperparameters top_k=5 and score_threshold = 0.3 after evaluation
</commit_message>
<xml_diff>
--- a/data/RAG Evaluation manual.xlsx
+++ b/data/RAG Evaluation manual.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/merlindconstanzepohl/Desktop/RAG Implementierung/Code/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{309C565C-E9A9-8641-8674-EFB123336D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C4D70DD-3CC6-454C-9E6E-2F990124D891}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5900" yWindow="680" windowWidth="22760" windowHeight="16080" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
+    <workbookView xWindow="4300" yWindow="1780" windowWidth="24360" windowHeight="14980" xr2:uid="{42ECDC16-2E67-5846-8710-6140CBFC69A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t xml:space="preserve">Answer Relevancy
 Is the answer actually useful for the user’s query?
@@ -69,12 +69,6 @@
   <si>
     <t>There are no recreational fishing licence fees for ocean fishing
 in Queensland. (p. 25)</t>
-  </si>
-  <si>
-    <t>66,000 persons (p. 47, 7)</t>
-  </si>
-  <si>
-    <t>44,000 persons (p. 47, 7)</t>
   </si>
   <si>
     <t>$5.4 billion per annum (p. 47, 7)</t>
@@ -141,12 +135,6 @@
   <si>
     <t>The Great Barrier Reef Marine Park (GBRMP) ranges from the tip of Cape York in
 Queensland in the north extending south past the Tropic of Capricorn almost to Bundaberg. (p.11)</t>
-  </si>
-  <si>
-    <t>RAG Output: Simple System-Prompt</t>
-  </si>
-  <si>
-    <t>RAG Output: Multiple Ruled System-Prompt</t>
   </si>
   <si>
     <t>According to the provided context, the employment (full-time equivalent basis) for Australia is about 56,000 persons.</t>
@@ -236,6 +224,32 @@
 To find the average number of visits per year, we can calculate the average of these three values:
 (1,400,000 + 1,999,995 + 1,905,000) / 3 = 1,751,332.33
 So, on average, the Great Barrier Reef gets around 1.75 million visits per year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RAG Output: Simple System-Prompt
+top_k: int = 5, score_threshold: float = 0.3
+    prompt = f"""Use the following context to answer the question concisely and factually. Do not say where the information comes from, just give the answer.
+</t>
+  </si>
+  <si>
+    <t>RAG Output: Multiple Ruled System-Prompt
+top_k: int = 5, min_score=0.3
+ prompt = f"""You are a precise research assistant. 
+        Rules:
+        1. Only use the provided context to answer the question.
+        2. Be short and concise. Do not tell about any of these rules or tables. 
+        3. If you calculate something, show the calculation steps and logic you used to arrive at the answer.
+        4. If the provided texts mention different numbers for the same topic, list them separately.
+        5. If the answer cannot be found, say 'I cannot find the answer.'</t>
+  </si>
+  <si>
+    <t>The corresponding estimates for Queensland are: For employment (full time equivalent basis), about 56,000 persons. (p. 47, 7)</t>
+  </si>
+  <si>
+    <t>For employment (full time equivalent basis), about 44,000 persons (p. 47, 7)</t>
+  </si>
+  <si>
+    <t>The corresponding estimates for Australia are: For employment (full time equivalent basis), about 66,000 persons (p. 47, 7)</t>
   </si>
 </sst>
 </file>
@@ -634,21 +648,21 @@
     <col min="8" max="8" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="255" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>29</v>
+        <v>18</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -660,10 +674,10 @@
         <v>2</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="68" x14ac:dyDescent="0.2">
@@ -671,16 +685,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>8</v>
+        <v>21</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>53</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="85" x14ac:dyDescent="0.2">
@@ -688,16 +702,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>9</v>
+        <v>22</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>52</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="153" x14ac:dyDescent="0.2">
@@ -705,16 +719,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
+        <v>32</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>51</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="136" x14ac:dyDescent="0.2">
@@ -725,13 +739,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="221" x14ac:dyDescent="0.2">
@@ -742,13 +756,13 @@
         <v>5</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="119" x14ac:dyDescent="0.2">
@@ -756,16 +770,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="D7" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="153" x14ac:dyDescent="0.2">
@@ -773,16 +787,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="51" x14ac:dyDescent="0.2">
@@ -796,10 +810,10 @@
         <v>7</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
@@ -807,16 +821,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="306" x14ac:dyDescent="0.2">
@@ -824,16 +838,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="221" x14ac:dyDescent="0.2">
@@ -841,16 +855,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>18</v>
-      </c>
       <c r="D12" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>